<commit_message>
Mejoras de datos de transaccion y fix kardex y exportaciones
</commit_message>
<xml_diff>
--- a/public/templates/plantilla_kardex_general.xlsx
+++ b/public/templates/plantilla_kardex_general.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rodnn\OneDrive\Desktop\Rodaltfl_dev_new\Proyects\sistema_de_inventario_multitenant_rengifo_v2\public\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rengifo\Desktop\Proyectos\sistema_de_inventario-rengifo-ltda\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8E65654-D37B-430C-B3F4-CFCA8220069D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{780C8AA4-C6AA-4A33-AF82-79A9E7E17411}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A2BCA4EF-8132-4769-A60E-E5566B4024F3}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A2BCA4EF-8132-4769-A60E-E5566B4024F3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -131,7 +131,7 @@
     <numFmt numFmtId="165" formatCode="#,##0_ ;[Red]\-#,##0\ "/>
     <numFmt numFmtId="166" formatCode="#,##0.00000"/>
   </numFmts>
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -272,6 +272,14 @@
       <name val="Arial Narrow"/>
       <family val="2"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -494,7 +502,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="94">
+  <cellXfs count="95">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -633,14 +641,32 @@
     <xf numFmtId="4" fontId="18" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="4" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="17" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="15" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="15" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -657,60 +683,42 @@
     <xf numFmtId="3" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="15" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="15" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="19" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -723,30 +731,31 @@
     <xf numFmtId="0" fontId="15" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="15" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="15" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="15" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="3" fontId="15" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="15" fillId="4" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="15" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="15" fillId="4" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="3" fontId="15" fillId="4" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="15" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="15" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="15" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1326,7 +1335,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1643,25 +1652,25 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3589914E-774A-4951-9B20-F2616ED98054}">
   <dimension ref="A1:O20"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="26.88671875" customWidth="1"/>
-    <col min="5" max="5" width="19.6640625" customWidth="1"/>
-    <col min="6" max="6" width="15.44140625" customWidth="1"/>
-    <col min="9" max="9" width="11.109375" customWidth="1"/>
-    <col min="10" max="10" width="11.33203125" customWidth="1"/>
-    <col min="11" max="11" width="12.44140625" customWidth="1"/>
-    <col min="12" max="12" width="11.77734375" customWidth="1"/>
-    <col min="13" max="13" width="11.109375" customWidth="1"/>
-    <col min="14" max="14" width="10.5546875" customWidth="1"/>
+    <col min="4" max="4" width="26.85546875" customWidth="1"/>
+    <col min="5" max="5" width="19.7109375" customWidth="1"/>
+    <col min="6" max="6" width="15.42578125" customWidth="1"/>
+    <col min="9" max="9" width="11.140625" customWidth="1"/>
+    <col min="10" max="10" width="11.28515625" customWidth="1"/>
+    <col min="11" max="11" width="12.42578125" customWidth="1"/>
+    <col min="12" max="12" width="11.7109375" customWidth="1"/>
+    <col min="13" max="13" width="11.140625" customWidth="1"/>
+    <col min="14" max="14" width="10.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="23.4" x14ac:dyDescent="0.3">
-      <c r="B1" s="73" t="s">
+    <row r="1" spans="1:15" ht="24" x14ac:dyDescent="0.25">
+      <c r="B1" s="56" t="s">
         <v>20</v>
       </c>
-      <c r="C1" s="73"/>
-      <c r="D1" s="73"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
       <c r="E1" s="1"/>
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
@@ -1672,13 +1681,13 @@
       <c r="L1" s="4"/>
       <c r="M1" s="4"/>
     </row>
-    <row r="2" spans="1:15" ht="25.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:15" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A2" s="5"/>
-      <c r="B2" s="74" t="s">
+      <c r="B2" s="57" t="s">
         <v>21</v>
       </c>
-      <c r="C2" s="74"/>
-      <c r="D2" s="74"/>
+      <c r="C2" s="57"/>
+      <c r="D2" s="57"/>
       <c r="E2" s="1"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
@@ -1689,13 +1698,13 @@
       <c r="L2" s="3"/>
       <c r="M2" s="3"/>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="6"/>
-      <c r="B3" s="75" t="s">
+      <c r="B3" s="58" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="75"/>
-      <c r="D3" s="75"/>
+      <c r="C3" s="58"/>
+      <c r="D3" s="58"/>
       <c r="E3" s="1"/>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
@@ -1706,63 +1715,63 @@
       <c r="L3" s="4"/>
       <c r="M3" s="4"/>
     </row>
-    <row r="4" spans="1:15" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="B4" s="76"/>
-      <c r="C4" s="76"/>
-      <c r="D4" s="76"/>
-      <c r="E4" s="56" t="s">
+    <row r="4" spans="1:15" ht="18" x14ac:dyDescent="0.25">
+      <c r="B4" s="59"/>
+      <c r="C4" s="59"/>
+      <c r="D4" s="59"/>
+      <c r="E4" s="73" t="s">
         <v>1</v>
       </c>
-      <c r="F4" s="56"/>
-      <c r="G4" s="56"/>
-      <c r="H4" s="56"/>
-      <c r="I4" s="56"/>
-      <c r="J4" s="56"/>
+      <c r="F4" s="73"/>
+      <c r="G4" s="73"/>
+      <c r="H4" s="73"/>
+      <c r="I4" s="73"/>
+      <c r="J4" s="73"/>
       <c r="K4" s="36"/>
       <c r="L4" s="3"/>
       <c r="M4" s="3"/>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="7"/>
-      <c r="B5" s="77" t="s">
+      <c r="B5" s="60" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="77"/>
-      <c r="D5" s="77"/>
-      <c r="E5" s="57" t="s">
+      <c r="C5" s="60"/>
+      <c r="D5" s="60"/>
+      <c r="E5" s="74" t="s">
         <v>19</v>
       </c>
-      <c r="F5" s="57"/>
-      <c r="G5" s="57"/>
-      <c r="H5" s="57"/>
-      <c r="I5" s="57"/>
-      <c r="J5" s="57"/>
+      <c r="F5" s="74"/>
+      <c r="G5" s="74"/>
+      <c r="H5" s="74"/>
+      <c r="I5" s="74"/>
+      <c r="J5" s="74"/>
       <c r="K5" s="37"/>
       <c r="L5" s="3"/>
       <c r="M5" s="3"/>
     </row>
-    <row r="6" spans="1:15" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:15" ht="18" x14ac:dyDescent="0.25">
       <c r="A6" s="8"/>
-      <c r="B6" s="60"/>
-      <c r="C6" s="60"/>
-      <c r="D6" s="60"/>
-      <c r="E6" s="58" t="s">
+      <c r="B6" s="66"/>
+      <c r="C6" s="66"/>
+      <c r="D6" s="66"/>
+      <c r="E6" s="75" t="s">
         <v>3</v>
       </c>
-      <c r="F6" s="58"/>
-      <c r="G6" s="58"/>
-      <c r="H6" s="58"/>
-      <c r="I6" s="58"/>
-      <c r="J6" s="58"/>
+      <c r="F6" s="75"/>
+      <c r="G6" s="75"/>
+      <c r="H6" s="75"/>
+      <c r="I6" s="75"/>
+      <c r="J6" s="75"/>
       <c r="K6" s="2"/>
       <c r="L6" s="10"/>
       <c r="M6" s="10"/>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="8"/>
-      <c r="B7" s="60"/>
-      <c r="C7" s="60"/>
-      <c r="D7" s="60"/>
+      <c r="B7" s="66"/>
+      <c r="C7" s="66"/>
+      <c r="D7" s="66"/>
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
       <c r="G7" s="1"/>
@@ -1773,7 +1782,7 @@
       <c r="L7" s="12"/>
       <c r="M7" s="12"/>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="9"/>
       <c r="B8" s="9"/>
       <c r="C8" s="9"/>
@@ -1787,81 +1796,82 @@
       <c r="K8" s="13"/>
       <c r="L8" s="13"/>
       <c r="M8" s="13"/>
+      <c r="N8" s="94"/>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A9" s="66" t="s">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A9" s="70" t="s">
         <v>4</v>
       </c>
-      <c r="B9" s="66"/>
-      <c r="C9" s="66"/>
+      <c r="B9" s="70"/>
+      <c r="C9" s="70"/>
       <c r="D9" s="14"/>
       <c r="E9" s="15"/>
       <c r="F9" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="G9" s="62"/>
-      <c r="H9" s="62"/>
-      <c r="I9" s="62"/>
-      <c r="J9" s="62"/>
+      <c r="G9" s="68"/>
+      <c r="H9" s="68"/>
+      <c r="I9" s="68"/>
+      <c r="J9" s="68"/>
       <c r="K9" s="34"/>
       <c r="L9" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="M9" s="61"/>
-      <c r="N9" s="61"/>
+      <c r="M9" s="67"/>
+      <c r="N9" s="67"/>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A10" s="67"/>
-      <c r="B10" s="67"/>
-      <c r="C10" s="67"/>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A10" s="71"/>
+      <c r="B10" s="71"/>
+      <c r="C10" s="71"/>
       <c r="D10" s="14"/>
       <c r="E10" s="15"/>
       <c r="F10" s="14"/>
-      <c r="G10" s="62"/>
-      <c r="H10" s="62"/>
-      <c r="I10" s="62"/>
-      <c r="J10" s="62"/>
+      <c r="G10" s="68"/>
+      <c r="H10" s="68"/>
+      <c r="I10" s="68"/>
+      <c r="J10" s="68"/>
       <c r="K10" s="34"/>
       <c r="L10" s="18"/>
       <c r="M10" s="19"/>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="B11" s="59"/>
-      <c r="C11" s="59"/>
-      <c r="D11" s="59"/>
+      <c r="B11" s="65"/>
+      <c r="C11" s="65"/>
+      <c r="D11" s="65"/>
       <c r="E11" s="14"/>
       <c r="F11" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="G11" s="68"/>
-      <c r="H11" s="68"/>
-      <c r="I11" s="68"/>
-      <c r="J11" s="68"/>
+      <c r="G11" s="72"/>
+      <c r="H11" s="72"/>
+      <c r="I11" s="72"/>
+      <c r="J11" s="72"/>
       <c r="K11" s="18"/>
-      <c r="L11" s="63" t="s">
+      <c r="L11" s="69" t="s">
         <v>9</v>
       </c>
-      <c r="M11" s="63"/>
+      <c r="M11" s="69"/>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="14"/>
       <c r="B12" s="22"/>
       <c r="C12" s="22"/>
       <c r="D12" s="22"/>
       <c r="E12" s="14"/>
       <c r="F12" s="20"/>
-      <c r="G12" s="68"/>
-      <c r="H12" s="68"/>
-      <c r="I12" s="68"/>
-      <c r="J12" s="68"/>
+      <c r="G12" s="72"/>
+      <c r="H12" s="72"/>
+      <c r="I12" s="72"/>
+      <c r="J12" s="72"/>
       <c r="K12" s="23"/>
       <c r="L12" s="18"/>
       <c r="M12" s="18"/>
     </row>
-    <row r="13" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="E13" s="24"/>
       <c r="F13" s="24"/>
       <c r="G13" s="24"/>
@@ -1872,23 +1882,23 @@
       <c r="L13" s="25"/>
       <c r="M13" s="25"/>
     </row>
-    <row r="14" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="69" t="s">
+    <row r="14" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="61" t="s">
         <v>10</v>
       </c>
-      <c r="B14" s="69" t="s">
+      <c r="B14" s="61" t="s">
         <v>11</v>
       </c>
-      <c r="C14" s="71" t="s">
+      <c r="C14" s="63" t="s">
         <v>12</v>
       </c>
-      <c r="D14" s="71" t="s">
+      <c r="D14" s="63" t="s">
         <v>13</v>
       </c>
-      <c r="E14" s="71" t="s">
+      <c r="E14" s="63" t="s">
         <v>14</v>
       </c>
-      <c r="F14" s="64" t="s">
+      <c r="F14" s="80" t="s">
         <v>15</v>
       </c>
       <c r="G14" s="82" t="s">
@@ -1901,63 +1911,63 @@
       </c>
       <c r="K14" s="84"/>
       <c r="L14" s="84"/>
-      <c r="M14" s="91" t="s">
+      <c r="M14" s="87" t="s">
         <v>24</v>
       </c>
-      <c r="N14" s="91"/>
+      <c r="N14" s="87"/>
       <c r="O14" s="47"/>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A15" s="70"/>
-      <c r="B15" s="70"/>
-      <c r="C15" s="72"/>
-      <c r="D15" s="72"/>
-      <c r="E15" s="72"/>
-      <c r="F15" s="65"/>
-      <c r="G15" s="78" t="s">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A15" s="62"/>
+      <c r="B15" s="62"/>
+      <c r="C15" s="64"/>
+      <c r="D15" s="64"/>
+      <c r="E15" s="64"/>
+      <c r="F15" s="81"/>
+      <c r="G15" s="76" t="s">
         <v>22</v>
       </c>
-      <c r="H15" s="78" t="s">
+      <c r="H15" s="76" t="s">
         <v>16</v>
       </c>
-      <c r="I15" s="80" t="s">
+      <c r="I15" s="78" t="s">
         <v>23</v>
       </c>
       <c r="J15" s="85" t="s">
         <v>22</v>
       </c>
-      <c r="K15" s="86" t="s">
+      <c r="K15" s="90" t="s">
         <v>16</v>
       </c>
-      <c r="L15" s="87" t="s">
+      <c r="L15" s="92" t="s">
         <v>23</v>
       </c>
-      <c r="M15" s="92" t="s">
+      <c r="M15" s="88" t="s">
         <v>24</v>
       </c>
-      <c r="N15" s="92" t="s">
+      <c r="N15" s="88" t="s">
         <v>23</v>
       </c>
       <c r="O15" s="48"/>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A16" s="70"/>
-      <c r="B16" s="70"/>
-      <c r="C16" s="72"/>
-      <c r="D16" s="72"/>
-      <c r="E16" s="72"/>
-      <c r="F16" s="65"/>
-      <c r="G16" s="79"/>
-      <c r="H16" s="79"/>
-      <c r="I16" s="81"/>
-      <c r="J16" s="88"/>
-      <c r="K16" s="89"/>
-      <c r="L16" s="90"/>
-      <c r="M16" s="93"/>
-      <c r="N16" s="93"/>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A16" s="62"/>
+      <c r="B16" s="62"/>
+      <c r="C16" s="64"/>
+      <c r="D16" s="64"/>
+      <c r="E16" s="64"/>
+      <c r="F16" s="81"/>
+      <c r="G16" s="77"/>
+      <c r="H16" s="77"/>
+      <c r="I16" s="79"/>
+      <c r="J16" s="86"/>
+      <c r="K16" s="91"/>
+      <c r="L16" s="93"/>
+      <c r="M16" s="89"/>
+      <c r="N16" s="89"/>
       <c r="O16" s="48"/>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17" s="49"/>
       <c r="B17" s="50"/>
       <c r="C17" s="51"/>
@@ -1975,7 +1985,7 @@
       <c r="M17" s="53"/>
       <c r="N17" s="53"/>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18" s="49"/>
       <c r="B18" s="50"/>
       <c r="C18" s="51"/>
@@ -2009,7 +2019,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A19" s="38"/>
       <c r="B19" s="39"/>
       <c r="C19" s="40"/>
@@ -2025,7 +2035,7 @@
       <c r="M19" s="54"/>
       <c r="N19" s="54"/>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A20" s="26"/>
       <c r="B20" s="27"/>
       <c r="C20" s="28"/>
@@ -2043,24 +2053,11 @@
     </row>
   </sheetData>
   <mergeCells count="33">
-    <mergeCell ref="B1:D1"/>
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="A14:A16"/>
-    <mergeCell ref="B14:B16"/>
-    <mergeCell ref="C14:C16"/>
-    <mergeCell ref="D14:D16"/>
-    <mergeCell ref="E14:E16"/>
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="B6:D7"/>
-    <mergeCell ref="M9:N9"/>
-    <mergeCell ref="G9:J10"/>
-    <mergeCell ref="L11:M11"/>
-    <mergeCell ref="A9:C9"/>
-    <mergeCell ref="A10:C10"/>
-    <mergeCell ref="G11:J12"/>
+    <mergeCell ref="M14:N14"/>
+    <mergeCell ref="M15:M16"/>
+    <mergeCell ref="N15:N16"/>
+    <mergeCell ref="K15:K16"/>
+    <mergeCell ref="L15:L16"/>
     <mergeCell ref="E4:J4"/>
     <mergeCell ref="E5:J5"/>
     <mergeCell ref="E6:J6"/>
@@ -2071,19 +2068,32 @@
     <mergeCell ref="G14:I14"/>
     <mergeCell ref="J14:L14"/>
     <mergeCell ref="J15:J16"/>
-    <mergeCell ref="M14:N14"/>
-    <mergeCell ref="M15:M16"/>
-    <mergeCell ref="N15:N16"/>
-    <mergeCell ref="K15:K16"/>
-    <mergeCell ref="L15:L16"/>
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="B6:D7"/>
+    <mergeCell ref="M9:N9"/>
+    <mergeCell ref="G9:J10"/>
+    <mergeCell ref="L11:M11"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="G11:J12"/>
+    <mergeCell ref="A14:A16"/>
+    <mergeCell ref="B14:B16"/>
+    <mergeCell ref="C14:C16"/>
+    <mergeCell ref="D14:D16"/>
+    <mergeCell ref="E14:E16"/>
+    <mergeCell ref="B1:D1"/>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B5:D5"/>
   </mergeCells>
   <conditionalFormatting sqref="G17 G19:J20">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="landscape" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+  <pageMargins left="0" right="0" top="0.74803149606299213" bottom="0.35433070866141736" header="0.31496062992125984" footer="0.31496062992125984"/>
+  <pageSetup scale="77" orientation="landscape" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix modulo de Kardex, plantilla de exportacion y Mejoras de diseño y disposicion
</commit_message>
<xml_diff>
--- a/public/templates/plantilla_kardex_general.xlsx
+++ b/public/templates/plantilla_kardex_general.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rengifo\Desktop\Proyectos\sistema_de_inventario-rengifo-ltda\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{780C8AA4-C6AA-4A33-AF82-79A9E7E17411}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{420248E3-BB5C-469E-9ACE-178A19D93D59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A2BCA4EF-8132-4769-A60E-E5566B4024F3}"/>
   </bookViews>
@@ -131,7 +131,7 @@
     <numFmt numFmtId="165" formatCode="#,##0_ ;[Red]\-#,##0\ "/>
     <numFmt numFmtId="166" formatCode="#,##0.00000"/>
   </numFmts>
-  <fonts count="21" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -173,13 +173,6 @@
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="20"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -307,7 +300,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -364,31 +357,71 @@
       <diagonal/>
     </border>
     <border>
+      <left style="medium">
+        <color theme="0"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="0"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color theme="0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
-        <color theme="0" tint="-0.24994659260841701"/>
+        <color theme="0"/>
       </left>
       <right style="thin">
-        <color theme="0" tint="-0.24994659260841701"/>
+        <color theme="0"/>
       </right>
-      <top style="hair">
-        <color indexed="64"/>
+      <top style="thin">
+        <color theme="0"/>
       </top>
-      <bottom style="hair">
-        <color indexed="64"/>
+      <bottom style="thin">
+        <color theme="0"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right style="medium">
+        <color theme="0"/>
+      </right>
+      <top style="medium">
+        <color theme="0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color theme="0"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
-        <color theme="0" tint="-0.24994659260841701"/>
+        <color theme="0"/>
       </left>
-      <right/>
-      <top style="hair">
-        <color indexed="64"/>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top style="thin">
+        <color theme="0"/>
       </top>
-      <bottom style="hair">
-        <color indexed="64"/>
-      </bottom>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -401,108 +434,29 @@
       <top style="thin">
         <color theme="1"/>
       </top>
-      <bottom style="thin">
-        <color theme="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="0" tint="-0.24994659260841701"/>
-      </left>
-      <right style="thin">
-        <color theme="0" tint="-0.24994659260841701"/>
-      </right>
-      <top/>
-      <bottom style="hair">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="0" tint="-0.24994659260841701"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="hair">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color theme="0"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color theme="0"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color theme="0"/>
-      </top>
       <bottom/>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color theme="0"/>
+        <color indexed="64"/>
       </left>
       <right style="thin">
-        <color theme="0"/>
+        <color indexed="64"/>
       </right>
       <top style="thin">
-        <color theme="0"/>
+        <color indexed="64"/>
       </top>
       <bottom style="thin">
-        <color theme="0"/>
+        <color indexed="64"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color theme="0"/>
-      </right>
-      <top style="medium">
-        <color theme="0"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color theme="0"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="0"/>
-      </left>
-      <right style="thin">
-        <color theme="0"/>
-      </right>
-      <top style="thin">
-        <color theme="0"/>
-      </top>
-      <bottom/>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="95">
+  <cellXfs count="88">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -510,252 +464,227 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="3" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="3" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="3" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="3" fontId="14" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="14" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="14" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="14" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="14" fillId="4" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="14" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="14" fillId="4" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="14" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="3" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="3" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="17" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="17" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="17" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="16" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="16" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="17" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="17" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="17" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="16" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="16" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="4" fontId="18" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="4" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="17" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="14" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="14" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="15" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="15" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="15" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="15" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="15" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="15" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="15" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="15" fillId="4" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="15" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="15" fillId="4" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="16" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="4" fontId="17" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="16" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="4" fontId="17" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -838,7 +767,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -893,7 +822,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -948,7 +877,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -1003,7 +932,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -1058,7 +987,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -1113,7 +1042,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -1168,7 +1097,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -1223,7 +1152,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -1278,7 +1207,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -1666,11 +1595,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="24" x14ac:dyDescent="0.25">
-      <c r="B1" s="56" t="s">
+      <c r="A1" s="60" t="s">
         <v>20</v>
       </c>
-      <c r="C1" s="56"/>
-      <c r="D1" s="56"/>
+      <c r="B1" s="60"/>
+      <c r="C1" s="60"/>
+      <c r="D1" s="60"/>
       <c r="E1" s="1"/>
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
@@ -1681,13 +1611,13 @@
       <c r="L1" s="4"/>
       <c r="M1" s="4"/>
     </row>
-    <row r="2" spans="1:15" ht="26.25" x14ac:dyDescent="0.25">
-      <c r="A2" s="5"/>
-      <c r="B2" s="57" t="s">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A2" s="61" t="s">
         <v>21</v>
       </c>
-      <c r="C2" s="57"/>
-      <c r="D2" s="57"/>
+      <c r="B2" s="61"/>
+      <c r="C2" s="61"/>
+      <c r="D2" s="61"/>
       <c r="E2" s="1"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
@@ -1699,12 +1629,12 @@
       <c r="M2" s="3"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A3" s="6"/>
-      <c r="B3" s="58" t="s">
+      <c r="A3" s="62" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="58"/>
-      <c r="D3" s="58"/>
+      <c r="B3" s="62"/>
+      <c r="C3" s="62"/>
+      <c r="D3" s="62"/>
       <c r="E3" s="1"/>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
@@ -1716,348 +1646,362 @@
       <c r="M3" s="4"/>
     </row>
     <row r="4" spans="1:15" ht="18" x14ac:dyDescent="0.25">
-      <c r="B4" s="59"/>
-      <c r="C4" s="59"/>
-      <c r="D4" s="59"/>
-      <c r="E4" s="73" t="s">
+      <c r="A4" s="86"/>
+      <c r="B4" s="86"/>
+      <c r="C4" s="86"/>
+      <c r="D4" s="86"/>
+      <c r="E4" s="35" t="s">
         <v>1</v>
       </c>
-      <c r="F4" s="73"/>
-      <c r="G4" s="73"/>
-      <c r="H4" s="73"/>
-      <c r="I4" s="73"/>
-      <c r="J4" s="73"/>
-      <c r="K4" s="36"/>
+      <c r="F4" s="35"/>
+      <c r="G4" s="35"/>
+      <c r="H4" s="35"/>
+      <c r="I4" s="35"/>
+      <c r="J4" s="35"/>
+      <c r="K4" s="23"/>
       <c r="L4" s="3"/>
       <c r="M4" s="3"/>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A5" s="7"/>
-      <c r="B5" s="60" t="s">
+      <c r="A5" s="63" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="60"/>
-      <c r="D5" s="60"/>
-      <c r="E5" s="74" t="s">
+      <c r="B5" s="63"/>
+      <c r="C5" s="63"/>
+      <c r="D5" s="63"/>
+      <c r="E5" s="36" t="s">
         <v>19</v>
       </c>
-      <c r="F5" s="74"/>
-      <c r="G5" s="74"/>
-      <c r="H5" s="74"/>
-      <c r="I5" s="74"/>
-      <c r="J5" s="74"/>
-      <c r="K5" s="37"/>
+      <c r="F5" s="36"/>
+      <c r="G5" s="36"/>
+      <c r="H5" s="36"/>
+      <c r="I5" s="36"/>
+      <c r="J5" s="36"/>
+      <c r="K5" s="24"/>
       <c r="L5" s="3"/>
       <c r="M5" s="3"/>
     </row>
     <row r="6" spans="1:15" ht="18" x14ac:dyDescent="0.25">
-      <c r="A6" s="8"/>
-      <c r="B6" s="66"/>
-      <c r="C6" s="66"/>
-      <c r="D6" s="66"/>
-      <c r="E6" s="75" t="s">
+      <c r="A6" s="87"/>
+      <c r="B6" s="87"/>
+      <c r="C6" s="87"/>
+      <c r="D6" s="87"/>
+      <c r="E6" s="37" t="s">
         <v>3</v>
       </c>
-      <c r="F6" s="75"/>
-      <c r="G6" s="75"/>
-      <c r="H6" s="75"/>
-      <c r="I6" s="75"/>
-      <c r="J6" s="75"/>
+      <c r="F6" s="37"/>
+      <c r="G6" s="37"/>
+      <c r="H6" s="37"/>
+      <c r="I6" s="37"/>
+      <c r="J6" s="37"/>
       <c r="K6" s="2"/>
-      <c r="L6" s="10"/>
-      <c r="M6" s="10"/>
+      <c r="L6" s="6"/>
+      <c r="M6" s="6"/>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A7" s="8"/>
-      <c r="B7" s="66"/>
-      <c r="C7" s="66"/>
-      <c r="D7" s="66"/>
+      <c r="A7" s="87"/>
+      <c r="B7" s="87"/>
+      <c r="C7" s="87"/>
+      <c r="D7" s="87"/>
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
       <c r="G7" s="1"/>
       <c r="H7" s="1"/>
       <c r="I7" s="1"/>
       <c r="J7" s="1"/>
-      <c r="K7" s="11"/>
-      <c r="L7" s="12"/>
-      <c r="M7" s="12"/>
+      <c r="K7" s="7"/>
+      <c r="L7" s="8"/>
+      <c r="M7" s="8"/>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A8" s="9"/>
-      <c r="B8" s="9"/>
-      <c r="C8" s="9"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="9"/>
+      <c r="A8" s="5"/>
+      <c r="B8" s="5"/>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
       <c r="F8" s="1"/>
       <c r="G8" s="1"/>
       <c r="H8" s="1"/>
       <c r="I8" s="1"/>
-      <c r="J8" s="9"/>
-      <c r="K8" s="13"/>
-      <c r="L8" s="13"/>
-      <c r="M8" s="13"/>
-      <c r="N8" s="94"/>
+      <c r="J8" s="5"/>
+      <c r="K8" s="9"/>
+      <c r="L8" s="9"/>
+      <c r="M8" s="9"/>
+      <c r="N8" s="27"/>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A9" s="70" t="s">
+      <c r="A9" s="53" t="s">
         <v>4</v>
       </c>
-      <c r="B9" s="70"/>
-      <c r="C9" s="70"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="15"/>
-      <c r="F9" s="16" t="s">
+      <c r="B9" s="53"/>
+      <c r="C9" s="53"/>
+      <c r="D9" s="10"/>
+      <c r="E9" s="11"/>
+      <c r="F9" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="G9" s="68"/>
-      <c r="H9" s="68"/>
-      <c r="I9" s="68"/>
-      <c r="J9" s="68"/>
-      <c r="K9" s="34"/>
-      <c r="L9" s="17" t="s">
+      <c r="G9" s="51"/>
+      <c r="H9" s="51"/>
+      <c r="I9" s="51"/>
+      <c r="J9" s="51"/>
+      <c r="K9" s="22"/>
+      <c r="L9" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="M9" s="67"/>
-      <c r="N9" s="67"/>
+      <c r="M9" s="50"/>
+      <c r="N9" s="50"/>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A10" s="71"/>
-      <c r="B10" s="71"/>
-      <c r="C10" s="71"/>
-      <c r="D10" s="14"/>
-      <c r="E10" s="15"/>
-      <c r="F10" s="14"/>
-      <c r="G10" s="68"/>
-      <c r="H10" s="68"/>
-      <c r="I10" s="68"/>
-      <c r="J10" s="68"/>
-      <c r="K10" s="34"/>
-      <c r="L10" s="18"/>
-      <c r="M10" s="19"/>
+      <c r="A10" s="54"/>
+      <c r="B10" s="54"/>
+      <c r="C10" s="54"/>
+      <c r="D10" s="10"/>
+      <c r="E10" s="11"/>
+      <c r="F10" s="10"/>
+      <c r="G10" s="51"/>
+      <c r="H10" s="51"/>
+      <c r="I10" s="51"/>
+      <c r="J10" s="51"/>
+      <c r="K10" s="22"/>
+      <c r="L10" s="14"/>
+      <c r="M10" s="15"/>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A11" s="20" t="s">
+      <c r="A11" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="B11" s="65"/>
-      <c r="C11" s="65"/>
-      <c r="D11" s="65"/>
-      <c r="E11" s="14"/>
-      <c r="F11" s="21" t="s">
+      <c r="B11" s="49"/>
+      <c r="C11" s="49"/>
+      <c r="D11" s="49"/>
+      <c r="E11" s="10"/>
+      <c r="F11" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="G11" s="72"/>
-      <c r="H11" s="72"/>
-      <c r="I11" s="72"/>
-      <c r="J11" s="72"/>
-      <c r="K11" s="18"/>
-      <c r="L11" s="69" t="s">
+      <c r="G11" s="55"/>
+      <c r="H11" s="55"/>
+      <c r="I11" s="55"/>
+      <c r="J11" s="55"/>
+      <c r="K11" s="14"/>
+      <c r="L11" s="52" t="s">
         <v>9</v>
       </c>
-      <c r="M11" s="69"/>
+      <c r="M11" s="52"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A12" s="14"/>
-      <c r="B12" s="22"/>
-      <c r="C12" s="22"/>
-      <c r="D12" s="22"/>
-      <c r="E12" s="14"/>
-      <c r="F12" s="20"/>
-      <c r="G12" s="72"/>
-      <c r="H12" s="72"/>
-      <c r="I12" s="72"/>
-      <c r="J12" s="72"/>
-      <c r="K12" s="23"/>
-      <c r="L12" s="18"/>
-      <c r="M12" s="18"/>
+      <c r="A12" s="10"/>
+      <c r="B12" s="18"/>
+      <c r="C12" s="18"/>
+      <c r="D12" s="18"/>
+      <c r="E12" s="10"/>
+      <c r="F12" s="16"/>
+      <c r="G12" s="55"/>
+      <c r="H12" s="55"/>
+      <c r="I12" s="55"/>
+      <c r="J12" s="55"/>
+      <c r="K12" s="19"/>
+      <c r="L12" s="14"/>
+      <c r="M12" s="14"/>
     </row>
     <row r="13" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="E13" s="24"/>
-      <c r="F13" s="24"/>
-      <c r="G13" s="24"/>
-      <c r="H13" s="24"/>
-      <c r="I13" s="24"/>
-      <c r="J13" s="24"/>
-      <c r="K13" s="25"/>
-      <c r="L13" s="25"/>
-      <c r="M13" s="25"/>
+      <c r="E13" s="20"/>
+      <c r="F13" s="20"/>
+      <c r="G13" s="20"/>
+      <c r="H13" s="20"/>
+      <c r="I13" s="20"/>
+      <c r="J13" s="20"/>
+      <c r="K13" s="21"/>
+      <c r="L13" s="21"/>
+      <c r="M13" s="21"/>
     </row>
     <row r="14" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="61" t="s">
+      <c r="A14" s="56" t="s">
         <v>10</v>
       </c>
-      <c r="B14" s="61" t="s">
+      <c r="B14" s="56" t="s">
         <v>11</v>
       </c>
-      <c r="C14" s="63" t="s">
+      <c r="C14" s="58" t="s">
         <v>12</v>
       </c>
-      <c r="D14" s="63" t="s">
+      <c r="D14" s="58" t="s">
         <v>13</v>
       </c>
-      <c r="E14" s="63" t="s">
+      <c r="E14" s="58" t="s">
         <v>14</v>
       </c>
-      <c r="F14" s="80" t="s">
+      <c r="F14" s="42" t="s">
         <v>15</v>
       </c>
-      <c r="G14" s="82" t="s">
+      <c r="G14" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="H14" s="83"/>
-      <c r="I14" s="83"/>
-      <c r="J14" s="84" t="s">
+      <c r="H14" s="45"/>
+      <c r="I14" s="45"/>
+      <c r="J14" s="46" t="s">
         <v>18</v>
       </c>
-      <c r="K14" s="84"/>
-      <c r="L14" s="84"/>
-      <c r="M14" s="87" t="s">
+      <c r="K14" s="46"/>
+      <c r="L14" s="46"/>
+      <c r="M14" s="28" t="s">
         <v>24</v>
       </c>
-      <c r="N14" s="87"/>
-      <c r="O14" s="47"/>
+      <c r="N14" s="28"/>
+      <c r="O14" s="25"/>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15" s="62"/>
-      <c r="B15" s="62"/>
-      <c r="C15" s="64"/>
-      <c r="D15" s="64"/>
-      <c r="E15" s="64"/>
-      <c r="F15" s="81"/>
-      <c r="G15" s="76" t="s">
+      <c r="A15" s="57"/>
+      <c r="B15" s="57"/>
+      <c r="C15" s="59"/>
+      <c r="D15" s="59"/>
+      <c r="E15" s="59"/>
+      <c r="F15" s="43"/>
+      <c r="G15" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="H15" s="76" t="s">
+      <c r="H15" s="38" t="s">
         <v>16</v>
       </c>
-      <c r="I15" s="78" t="s">
+      <c r="I15" s="40" t="s">
         <v>23</v>
       </c>
-      <c r="J15" s="85" t="s">
+      <c r="J15" s="47" t="s">
         <v>22</v>
       </c>
-      <c r="K15" s="90" t="s">
+      <c r="K15" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="L15" s="92" t="s">
+      <c r="L15" s="33" t="s">
         <v>23</v>
       </c>
-      <c r="M15" s="88" t="s">
+      <c r="M15" s="29" t="s">
         <v>24</v>
       </c>
-      <c r="N15" s="88" t="s">
+      <c r="N15" s="29" t="s">
         <v>23</v>
       </c>
-      <c r="O15" s="48"/>
+      <c r="O15" s="26"/>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16" s="62"/>
-      <c r="B16" s="62"/>
-      <c r="C16" s="64"/>
-      <c r="D16" s="64"/>
-      <c r="E16" s="64"/>
-      <c r="F16" s="81"/>
-      <c r="G16" s="77"/>
-      <c r="H16" s="77"/>
-      <c r="I16" s="79"/>
-      <c r="J16" s="86"/>
-      <c r="K16" s="91"/>
-      <c r="L16" s="93"/>
-      <c r="M16" s="89"/>
-      <c r="N16" s="89"/>
-      <c r="O16" s="48"/>
+      <c r="A16" s="57"/>
+      <c r="B16" s="57"/>
+      <c r="C16" s="59"/>
+      <c r="D16" s="59"/>
+      <c r="E16" s="59"/>
+      <c r="F16" s="43"/>
+      <c r="G16" s="39"/>
+      <c r="H16" s="39"/>
+      <c r="I16" s="41"/>
+      <c r="J16" s="48"/>
+      <c r="K16" s="32"/>
+      <c r="L16" s="34"/>
+      <c r="M16" s="30"/>
+      <c r="N16" s="30"/>
+      <c r="O16" s="26"/>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A17" s="49"/>
-      <c r="B17" s="50"/>
-      <c r="C17" s="51"/>
-      <c r="D17" s="51"/>
-      <c r="E17" s="52"/>
-      <c r="F17" s="51"/>
-      <c r="G17" s="55">
+      <c r="A17" s="64"/>
+      <c r="B17" s="65"/>
+      <c r="C17" s="66"/>
+      <c r="D17" s="66"/>
+      <c r="E17" s="67"/>
+      <c r="F17" s="66"/>
+      <c r="G17" s="68">
         <v>0</v>
       </c>
-      <c r="H17" s="55"/>
-      <c r="I17" s="55"/>
-      <c r="J17" s="55"/>
-      <c r="K17" s="55"/>
-      <c r="L17" s="55"/>
-      <c r="M17" s="53"/>
-      <c r="N17" s="53"/>
+      <c r="H17" s="68"/>
+      <c r="I17" s="68"/>
+      <c r="J17" s="68"/>
+      <c r="K17" s="68"/>
+      <c r="L17" s="68"/>
+      <c r="M17" s="69"/>
+      <c r="N17" s="69"/>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A18" s="49"/>
-      <c r="B18" s="50"/>
-      <c r="C18" s="51"/>
-      <c r="D18" s="51"/>
-      <c r="E18" s="52"/>
-      <c r="F18" s="51" t="s">
+      <c r="A18" s="80"/>
+      <c r="B18" s="81"/>
+      <c r="C18" s="82"/>
+      <c r="D18" s="82"/>
+      <c r="E18" s="83"/>
+      <c r="F18" s="82" t="s">
         <v>25</v>
       </c>
-      <c r="G18" s="55">
+      <c r="G18" s="84">
         <v>0</v>
       </c>
-      <c r="H18" s="55" t="s">
+      <c r="H18" s="84" t="s">
         <v>26</v>
       </c>
-      <c r="I18" s="55">
+      <c r="I18" s="84">
         <v>0</v>
       </c>
-      <c r="J18" s="55">
+      <c r="J18" s="84">
         <v>0</v>
       </c>
-      <c r="K18" s="55" t="s">
+      <c r="K18" s="84" t="s">
         <v>26</v>
       </c>
-      <c r="L18" s="55">
+      <c r="L18" s="84">
         <v>0</v>
       </c>
-      <c r="M18" s="53" t="s">
+      <c r="M18" s="85" t="s">
         <v>26</v>
       </c>
-      <c r="N18" s="53">
+      <c r="N18" s="85">
         <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A19" s="38"/>
-      <c r="B19" s="39"/>
-      <c r="C19" s="40"/>
-      <c r="D19" s="40"/>
-      <c r="E19" s="41"/>
-      <c r="F19" s="40"/>
-      <c r="G19" s="42"/>
-      <c r="H19" s="42"/>
-      <c r="I19" s="43"/>
-      <c r="J19" s="44"/>
-      <c r="K19" s="45"/>
-      <c r="L19" s="46"/>
-      <c r="M19" s="54"/>
-      <c r="N19" s="54"/>
+      <c r="A19" s="70"/>
+      <c r="B19" s="71"/>
+      <c r="C19" s="72"/>
+      <c r="D19" s="72"/>
+      <c r="E19" s="73"/>
+      <c r="F19" s="72"/>
+      <c r="G19" s="74"/>
+      <c r="H19" s="74"/>
+      <c r="I19" s="75"/>
+      <c r="J19" s="76"/>
+      <c r="K19" s="77"/>
+      <c r="L19" s="78"/>
+      <c r="M19" s="79"/>
+      <c r="N19" s="79"/>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A20" s="26"/>
-      <c r="B20" s="27"/>
-      <c r="C20" s="28"/>
-      <c r="D20" s="28"/>
-      <c r="E20" s="29"/>
-      <c r="F20" s="28"/>
-      <c r="G20" s="30"/>
-      <c r="H20" s="30"/>
-      <c r="I20" s="31"/>
-      <c r="J20" s="32"/>
-      <c r="K20" s="33"/>
-      <c r="L20" s="35"/>
-      <c r="M20" s="54"/>
-      <c r="N20" s="54"/>
+      <c r="A20" s="70"/>
+      <c r="B20" s="71"/>
+      <c r="C20" s="72"/>
+      <c r="D20" s="72"/>
+      <c r="E20" s="73"/>
+      <c r="F20" s="72"/>
+      <c r="G20" s="74"/>
+      <c r="H20" s="74"/>
+      <c r="I20" s="75"/>
+      <c r="J20" s="76"/>
+      <c r="K20" s="77"/>
+      <c r="L20" s="78"/>
+      <c r="M20" s="79"/>
+      <c r="N20" s="79"/>
     </row>
   </sheetData>
   <mergeCells count="33">
-    <mergeCell ref="M14:N14"/>
-    <mergeCell ref="M15:M16"/>
-    <mergeCell ref="N15:N16"/>
-    <mergeCell ref="K15:K16"/>
-    <mergeCell ref="L15:L16"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A14:A16"/>
+    <mergeCell ref="B14:B16"/>
+    <mergeCell ref="C14:C16"/>
+    <mergeCell ref="D14:D16"/>
+    <mergeCell ref="E14:E16"/>
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="M9:N9"/>
+    <mergeCell ref="G9:J10"/>
+    <mergeCell ref="L11:M11"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="G11:J12"/>
+    <mergeCell ref="A6:D7"/>
     <mergeCell ref="E4:J4"/>
     <mergeCell ref="E5:J5"/>
     <mergeCell ref="E6:J6"/>
@@ -2068,24 +2012,11 @@
     <mergeCell ref="G14:I14"/>
     <mergeCell ref="J14:L14"/>
     <mergeCell ref="J15:J16"/>
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="B6:D7"/>
-    <mergeCell ref="M9:N9"/>
-    <mergeCell ref="G9:J10"/>
-    <mergeCell ref="L11:M11"/>
-    <mergeCell ref="A9:C9"/>
-    <mergeCell ref="A10:C10"/>
-    <mergeCell ref="G11:J12"/>
-    <mergeCell ref="A14:A16"/>
-    <mergeCell ref="B14:B16"/>
-    <mergeCell ref="C14:C16"/>
-    <mergeCell ref="D14:D16"/>
-    <mergeCell ref="E14:E16"/>
-    <mergeCell ref="B1:D1"/>
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="M14:N14"/>
+    <mergeCell ref="M15:M16"/>
+    <mergeCell ref="N15:N16"/>
+    <mergeCell ref="K15:K16"/>
+    <mergeCell ref="L15:L16"/>
   </mergeCells>
   <conditionalFormatting sqref="G17 G19:J20">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">

</xml_diff>